<commit_message>
Update UI styles and enhance scraping functionality
- Changed file permissions for run_ui.sh to executable.
- Updated UI styles in app/ui.py for improved aesthetics and responsiveness, including background gradients and layout adjustments.
- Added start_page parameter to scraping functions in pipeline modules to allow for more flexible pagination.
- Adjusted the handling of start_page in seoudi_graphql.py to ensure compatibility with existing URL parsing logic.
- Updated subcategories.xlsx with new data.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/catalog/subcategories.xlsx
+++ b/catalog/subcategories.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,7 +483,6 @@
           <t>أدوات مطبخ</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>adoat-mtbkh187</t>
@@ -515,7 +514,6 @@
           <t>بطاريات ولمبات</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>btaryat-olmbat188</t>
@@ -547,7 +545,6 @@
           <t>بلاستيك</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>blastyk189</t>
@@ -579,7 +576,6 @@
           <t>اكياس وحفظ طعام</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>akyas-ohfth-taaam190</t>
@@ -611,7 +607,6 @@
           <t>مكونات الطبخ</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>mkonat-altbkh191</t>
@@ -643,7 +638,6 @@
           <t>معلبات و برطمانات و غيرها</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>maalbat-o-brtmanat-o-ghyrha192</t>
@@ -675,7 +669,6 @@
           <t>بقوليات</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>bkolyat193</t>
@@ -707,7 +700,6 @@
           <t>زيوت و سمن</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>zyot-o-smn194</t>
@@ -739,7 +731,6 @@
           <t>صلصات و مخللات</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>mkhllat195</t>
@@ -771,7 +762,6 @@
           <t>أرز و مكرونة</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>arz-o-mkron196</t>
@@ -803,7 +793,6 @@
           <t>دقيق، مستلزمات خبز</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>dkyk-mstlzmat-khbz197</t>
@@ -835,7 +824,6 @@
           <t>منتجات الفطور الغذائية</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>mntgat-alftor-alghthayy198</t>
@@ -867,7 +855,6 @@
           <t>بطاطس و مقبلات</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>btats-o-mkblat199</t>
@@ -899,7 +886,6 @@
           <t>خضار مجمد</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>khdar-mgmd200</t>
@@ -931,7 +917,6 @@
           <t>بيتزا و فطائر</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>bytza-o-ftayr201</t>
@@ -963,7 +948,6 @@
           <t>وجبات جاهزة</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>ogbat-gahz202</t>
@@ -995,7 +979,6 @@
           <t>مشروبات غازيه</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>mshrobat-ghazyh203</t>
@@ -1027,7 +1010,6 @@
           <t>الشاي و القهوة</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>alshay-o-alkho204</t>
@@ -1059,7 +1041,6 @@
           <t>عصائر</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>aasayr205</t>
@@ -1091,7 +1072,6 @@
           <t>مياه</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>myah206</t>
@@ -1123,7 +1103,6 @@
           <t>مشروبات الطاقة</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>mshrobat-altak207</t>
@@ -1155,7 +1134,6 @@
           <t>توست</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>tost208</t>
@@ -1187,7 +1165,6 @@
           <t>معجنات</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>maagnat209</t>
@@ -1219,7 +1196,6 @@
           <t>كيك و حلويات</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>kyk-o-hloyat210</t>
@@ -1251,7 +1227,6 @@
           <t>شيكولاته</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>shykolath211</t>
@@ -1283,7 +1258,6 @@
           <t>البسكويت</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>albskoyt212</t>
@@ -1315,7 +1289,6 @@
           <t>الشيبسي و السناكس</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>alshybsy-o-alsnaks213</t>
@@ -1347,7 +1320,6 @@
           <t>الحلويات وكعك</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>alhloyat-okaak214</t>
@@ -1379,7 +1351,6 @@
           <t>المكسرات</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>almksrat215</t>
@@ -1411,7 +1382,6 @@
           <t>فواكه</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>foakh216</t>
@@ -1443,7 +1413,6 @@
           <t>خضروات</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>khdroat217</t>
@@ -1475,7 +1444,6 @@
           <t>تمور</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>tmor218</t>
@@ -1507,7 +1475,6 @@
           <t>مزيلات العرق</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>mzylat-alaark219</t>
@@ -1539,7 +1506,6 @@
           <t>العناية بالفم</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>alaanay-balfm220</t>
@@ -1571,7 +1537,6 @@
           <t>مزيلات عرق</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>mzylat-aark221</t>
@@ -1603,7 +1568,6 @@
           <t>عناية بالشعر</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>aanay-balshaar222</t>
@@ -1635,7 +1599,6 @@
           <t>عناية بالبشرة</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>aanay-balbshr223</t>
@@ -1667,7 +1630,6 @@
           <t>حفاضات</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>hfadat224</t>
@@ -1699,7 +1661,6 @@
           <t>أكل أطفال</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>akl-atfal225</t>
@@ -1731,7 +1692,6 @@
           <t>غسيل</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>ghsyl226</t>
@@ -1763,7 +1723,6 @@
           <t>جلي</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>gly227</t>
@@ -1795,7 +1754,6 @@
           <t>تنظيف أسطح</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>tnthyf-asth228</t>
@@ -1827,7 +1785,6 @@
           <t>مناديل ورقيات</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>mnadyl-orkyat229</t>
@@ -1859,7 +1816,6 @@
           <t>اللبن</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>allbn230</t>
@@ -1891,7 +1847,6 @@
           <t>زبادي</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>zbady231</t>
@@ -1923,7 +1878,6 @@
           <t>زبدة و كريمة</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>zbd-o-krym232</t>
@@ -1955,7 +1909,6 @@
           <t>بيض</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>byd233</t>
@@ -1987,7 +1940,6 @@
           <t>الجبنة واللبنة</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>algbn-oallbn234</t>
@@ -2003,6 +1955,26 @@
           <t>product_images</t>
         </is>
       </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" t="n">
+        <v>235</v>
+      </c>
+      <c r="C50" t="n">
+        <v>235</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>غير مصنف</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>